<commit_message>
Add guest roster support, attendance handling, flexible pairing for odd headcount, and README updates
</commit_message>
<xml_diff>
--- a/嘉宾偏好_第一轮.xlsx
+++ b/嘉宾偏好_第一轮.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mumark/Desktop/Documents/AI Startup/Claude Code/Dating_Match/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mumark/Desktop/Documents/AI_Startup/Claude_Code/Dating_Match/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A3EE79-53EA-7942-BAAF-4D916EA42890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA133E3-B4F2-AA4F-8C0E-AB2AC80CD74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7480" yWindow="4060" windowWidth="23960" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21760" yWindow="3700" windowWidth="23960" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="偏好" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="32">
   <si>
     <t>嘉宾类型</t>
   </si>
@@ -44,9 +44,6 @@
     <t>男</t>
   </si>
   <si>
-    <t>M11</t>
-  </si>
-  <si>
     <t>M2</t>
   </si>
   <si>
@@ -59,9 +56,6 @@
     <t>M10</t>
   </si>
   <si>
-    <t>M4</t>
-  </si>
-  <si>
     <t>M7</t>
   </si>
   <si>
@@ -71,15 +65,6 @@
     <t>F10</t>
   </si>
   <si>
-    <t>F12</t>
-  </si>
-  <si>
-    <t>F2</t>
-  </si>
-  <si>
-    <t>F11</t>
-  </si>
-  <si>
     <t>F4</t>
   </si>
   <si>
@@ -93,9 +78,6 @@
   </si>
   <si>
     <t>M3</t>
-  </si>
-  <si>
-    <t>M12</t>
   </si>
   <si>
     <t>M6</t>
@@ -502,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -528,10 +510,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -542,10 +524,10 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -556,10 +538,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -570,10 +552,10 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -584,10 +566,10 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -598,10 +580,10 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -612,10 +594,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -626,10 +608,10 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -640,10 +622,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -654,38 +636,38 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C12" t="s">
         <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -693,13 +675,13 @@
         <v>6</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -707,13 +689,13 @@
         <v>6</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -721,13 +703,13 @@
         <v>6</v>
       </c>
       <c r="B16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -735,13 +717,13 @@
         <v>6</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -749,13 +731,13 @@
         <v>6</v>
       </c>
       <c r="B18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -763,13 +745,13 @@
         <v>6</v>
       </c>
       <c r="B19">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -777,13 +759,13 @@
         <v>6</v>
       </c>
       <c r="B20">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -791,73 +773,18 @@
         <v>6</v>
       </c>
       <c r="B21">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>6</v>
-      </c>
-      <c r="B22">
-        <v>9</v>
-      </c>
-      <c r="C22" t="s">
-        <v>21</v>
-      </c>
-      <c r="D22" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23">
-        <v>10</v>
-      </c>
-      <c r="C23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24">
-        <v>11</v>
-      </c>
-      <c r="C24" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25">
-        <v>12</v>
-      </c>
-      <c r="C25" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -868,10 +795,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -879,7 +806,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -887,7 +814,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -895,7 +822,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -903,7 +830,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -911,15 +838,15 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
         <v>31</v>
-      </c>
-      <c r="B7" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>